<commit_message>
Add verified vendor candidates tab to the evaluation workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjwPqWZk3R28VRXPEjRwhw
</commit_message>
<xml_diff>
--- a/fleet-ops-starter/evaluacion-proveedores.xlsx
+++ b/fleet-ops-starter/evaluacion-proveedores.xlsx
@@ -9,11 +9,12 @@
   </bookViews>
   <sheets>
     <sheet name="Inicio" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Criterios" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Evaluación" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Costos" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Preguntas" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Piloto" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Candidatos" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Criterios" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Evaluación" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Costos" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Preguntas" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Piloto" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="352">
   <si>
     <t xml:space="preserve">Evaluación de proveedores de GPS y de rutas</t>
   </si>
@@ -36,6 +37,12 @@
     <t xml:space="preserve">Cómo usarla, paso a paso</t>
   </si>
   <si>
+    <t xml:space="preserve">0. Mira los candidatos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pestaña Candidatos resume más de una docena de proveedores con su contacto, lo que ofrecen y lo que falta confirmar. Elige 3 para empezar.</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Define criterios y pesos</t>
   </si>
   <si>
@@ -144,25 +151,25 @@
     <t xml:space="preserve">La decisión final se toma con el piloto y el costo, no con el puntaje solo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Candidatos para investigar (no son recomendaciones)</t>
+    <t xml:space="preserve">Candidatos (no son recomendaciones)</t>
   </si>
   <si>
     <t xml:space="preserve">GPS y telemática</t>
   </si>
   <si>
-    <t xml:space="preserve">Informac (producto Systrack, sobre la plataforma GpsGate; empresa dominicana), Geotab, Gurtam (Wialon, por distribuidores locales) y Samsara. La disponibilidad de Samsara en la República Dominicana no está confirmada.</t>
+    <t xml:space="preserve">Ver la pestaña Candidatos: proveedores dominicanos (GPS LINK, Ultron GPS, WolfTrak, proGPS, Multisol, Prosecon, Informac) y plataformas internacionales (Geotab, Wialon).</t>
   </si>
   <si>
     <t xml:space="preserve">Rutas y despacho</t>
   </si>
   <si>
-    <t xml:space="preserve">Routific (app del conductor en español desde febrero de 2026), OptimoRoute (app del conductor en español), Onfleet (para flotas propias de unos 3 a 50 vehículos).</t>
+    <t xml:space="preserve">Ver la pestaña Candidatos: SimpliRoute, Drivin, Routific, OptimoRoute y MotoConcho RD. Ninguno confirma presencia en la RD en su página.</t>
   </si>
   <si>
     <t xml:space="preserve">Aviso</t>
   </si>
   <si>
-    <t xml:space="preserve">Esta lista sale de una investigación general. No he evaluado a estos proveedores ni verificado precios o disponibilidad en la República Dominicana: confírmalo con cada uno.</t>
+    <t xml:space="preserve">La pestaña Candidatos recoge lo que dice cada empresa en su página, revisado el 09/10/2026. No he probado ni evaluado ningún producto, y casi ningún precio es público: confírmalo por escrito con cada uno.</t>
   </si>
   <si>
     <t xml:space="preserve">Colores y límites</t>
@@ -192,6 +199,351 @@
     <t xml:space="preserve">El puntaje mide lo que tú califiques. Si los criterios o los pesos no reflejan tu operación, el resultado tampoco lo hará. Revisa los pesos con tu jefe.</t>
   </si>
   <si>
+    <t xml:space="preserve">Candidatos a evaluar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datos tomados de las páginas oficiales de cada empresa y de búsquedas, revisados el 09/10/2026. Son lo que ellas dicen: nada está confirmado con el proveedor. Pide por escrito lo marcado como pendiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proveedor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contacto publicado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qué ofrece (según su página)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio publicado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente de confirmar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPS LINK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPS local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oficina en Santo Domingo. WhatsApp y teléfono +1 (305) 927-2739; info@gpslinkusa.com. Lun a vie 8:30 a 18:00; emergencias 24/7.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ubicación en tiempo real, recorridos, alertas, reportes, corte remoto de motor, botón de pánico, API para ERP. Planes Básico, Full y Corporativo. Opera en RD y Haití con SIM de varias operadoras (Claro, Altice, Digicel). Contrato corporativo desde 3 vehículos, con SLA a medida.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí: solución para motos y reparto (paradas, reportes por conductor, geocercas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web y móvil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No publica precios. "Consultar precio" más IVA por vehículo. Facturación anual con -20%; instalación sin costo en pago anual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precios, plazo y cancelación, modelo de equipo y garantía, razón social, cobertura en rutas largas. El teléfono de contacto es de Estados Unidos (+1 305): confirma que atienden en la RD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.gpslinkusa.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ultron GPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaza Bonaire, Av. San Vicente de Paúl 280, Santo Domingo Este. Tel. (809) 895-0273; WhatsApp 809-754-2056 (según el enlace); info@ultrongps.com. Lun a vie 8:30 a 17:30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rastreo en tiempo real, reportes en Excel y PDF, geocercas, mantenimiento por fechas o kilometraje, sensores (combustible, temperatura, conductor), optimización de rutas y entregas, centro de monitoreo 24/7 para emergencias. Instalación incluso fines de semana. Demostración gratuita.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mencionadas entre los tipos de vehículo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web y móvil (según un testimonio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No publica precios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precios, permanencia (solo el servicio de expansión indica contrato mensual sin penalidad), compatibilidad de equipos, cómo funciona la optimización de rutas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ultrongps.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WolfTrak Global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calle Los Pinos #3, Santo Domingo Este. Tel. +1 (829) 594-6821 y chat. Cotización en menos de 24 horas hábiles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rastreo para camiones y vehículos, geocercas, corte remoto, control de combustible, cámaras, calificación de conductores, API, alertas por WhatsApp, reportes por correo (CSV, Excel, PDF), historial de 1 año. Servicio técnico en varias ciudades (Santo Domingo, Santiago, La Romana, Higüey-Bávaro).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No confirmado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android e iOS, incluida en todos los planes; plataforma web en versión beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preguntas frecuentes: desde RD$600/mes más ITBIS para rastreo básico (equipo en renta). Sin lista de precios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motos, permanencia del contrato, razón social. Sus contadores en la página aparecen en cero y dice operar "desde 2013" mientras otras fuentes dicen 2014: no tomes sus cifras de clientes como verificadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://wolftrakglobal.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proGPS (Pro GPS &amp; Technology)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Av. Las Carreras, Edif. M-48, Apto. 1B, Santiago. Tel. (809) 276-2595 y (809) 924-7060. Lun a vie 8:00 a 18:00; sáb 8:00 a 12:00.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rastreo vehicular, logística de flotas, video telemática, servicios de campo. Alertas de conducción peligrosa, más de 15 tipos de reportes (XLS, PDF, CSV, TXT). Acceso web y apps. Dice tener más de 100 empresas clientes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android e iOS, y web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Ver planes", pero sin precios en la página.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motos, geocercas (solo menciona puntos de interés), precios, permanencia, correo y WhatsApp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://progps.com.do/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multisol GNP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ave. 1ra. No. 8, Jardines del Sur, Santo Domingo. Tel. (849) 289-0555 y (809) 757-0555; info@multisolgnp.com.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiempo real, apagado remoto, audio en vivo, historial, geocercas, alertas de velocidad, informes de rutas, paradas y combustible. Dos plataformas: NSWox (reportes detallados) y GPSDD (básica).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No mencionadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Móvil y web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motos, precios, permanencia, cobertura, instalación y garantía.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.multisolgnp.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prosecon Technology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calle Dolores Rodríguez Objío No. 1, Mirador Sur, Santo Domingo. Tel. +1 809-535-7094. Los números de WhatsApp y correo de la página son inconsistentes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rastreo de vehículos, camiones, autos y barcos en RD y Haití; apagado de motor, geocercas, puntos de interés, reportes. La información que revisé es de un artículo de julio de 2021.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plataforma web; app móvil no aparece</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si la información sigue vigente, motos, app móvil, precios, y el contacto correcto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://prosecon.tech/es/blog/rastreo-satelital-gps-vehiculos-republica-dominicana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informac (Systrack)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No encontré su sitio oficial ni su contacto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empresa dominicana de rastreo; Systrack funciona sobre la plataforma GpsGate con equipos Teltonika serie FMB. Según el blog de GpsGate (21/03/2024): unos 800 clientes de flotas y unos 23.000 vehículos. Geocercas, tiempo real y recuperación de vehículos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin información.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todo lo propio de la empresa: sitio, contacto, precios, planes. Las cifras vienen del proveedor de la plataforma, no de Informac.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://gpsgate.com/blog/global-collabs-gpsgate-informac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gps.do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensanche La Fe, Santo Domingo (según un buscador).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dice ofrecer rastreo satelital sin pagos mensuales ni contratos (según el resultado de búsqueda).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No verificado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No verificado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Su página no respondió al revisarla (error 503). Comprueba con cuidado qué incluye "sin pagos mensuales" antes de contratar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://gps.do/inicio/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geotab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPS internacional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin socio dominicano encontrado. Contactar a Geotab Latinoamérica.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plataforma de telemática con más de 300.000 suscripciones en Latinoamérica (abril de 2025). Su artículo sobre el Caribe (abril de 2025) no menciona la RD ni nombra distribuidores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin información pública.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si existe un distribuidor en la RD, su precio, soporte local y compatibilidad con motos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.geotab.com/es-latam/blog/gestion-de-flotas-caribe/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wialon (Gurtam)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin socio dominicano confirmado. Gurtam publica un mapa de socios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plataforma usada por muchos integradores en el mundo; en la búsqueda no apareció ningún socio dominicano. Es posible que algunas empresas locales la usen sin decirlo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si algún proveedor local la usa; se verifica en el mapa de socios de Gurtam o preguntando a cada empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://blog.gurtam.com/en/blog/top-20-international-gurtam-partners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SimpliRoute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rutas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formulario de ventas y solicitud de demo en su sitio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planificación de rutas con tráfico, ventanas horarias y bloqueo de zonas; app del conductor; ETA por correo, SMS o WhatsApp; gestión de flota. Prueba y herramienta gratuita para flotas de menos de 10 vehículos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App para conductores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No publica planes ni precios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si atienden en la RD, mapas y tráfico de Santo Domingo, motos, precios en pesos y soporte local. Su página no lista países ni nombra la RD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.simpliroute.com/es</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drivin (Descartes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formulario de demo y WhatsApp (enlace en su sitio).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMS con optimización de rutas con IA, torre de control, aviso de llegada al cliente, app del conductor con prueba de entrega, integraciones con ERP. Dice operar en "toda Latinoamérica".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App con prueba de entrega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobertura en la RD (no aparece), motos, precios y soporte local.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://driv.in/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Routific y OptimoRoute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vía sus sitios oficiales (demo o prueba).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software de rutas para flotas pequeñas. La app del conductor de Routific está en español desde febrero de 2026; la de OptimoRoute ofrece español entre sus idiomas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precios por vehículo o conductor al mes, que varían según la fuente. Confirma con cada empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si funcionan bien con los mapas y las direcciones de Santo Domingo, motos, y soporte en español.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.g2.com/compare/optimoroute-vs-routific</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MotoConcho RD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rutas / moto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sitio: motoconchord.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Según un resultado de búsqueda: app dominicana que organiza motoconchos, con seguimiento en vivo y plan básico de RD$500/mes. Parece pensada para motoconchos, no para flotas con rutas planificadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí, según la búsqueda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RD$500/mes plan básico, según la búsqueda (sin verificar).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todo: su sitio no respondió al revisarlo (error 503). Confirma si sirve para una flota propia de repartidores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://motoconchord.org/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cómo usar esta lista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Elige 3 candidatos y cópialos a los encabezados de Evaluación. Una mezcla útil: 2 de GPS local con soporte en la RD y 1 de rutas si lo necesitas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Para motos, pide primero a GPS LINK y Ultron GPS que muestren el equipo y la app en una moto real; los demás no lo confirman en su página.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Pide a cada uno la misma lista de Preguntas y precios por escrito.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Los candidatos de rutas no confirman presencia en la RD: pregunta antes de invertir tiempo en una demo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Un proveedor sin respuesta en dos días hábiles es información: el soporte antes de la venta suele ser el mejor que vas a recibir.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Criterios y pesos</t>
   </si>
   <si>
@@ -262,9 +614,6 @@
   </si>
   <si>
     <t xml:space="preserve">Ordena paradas, respeta horarios prometidos y permite varios tipos de vehículo. 1 = manual; 5 = automático y ajustable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rutas</t>
   </si>
   <si>
     <t xml:space="preserve">App del conductor en español y simple</t>
@@ -748,7 +1097,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
     <numFmt numFmtId="170" formatCode="0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -808,6 +1157,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <u val="single"/>
+      <sz val="9"/>
+      <color rgb="FF0563C1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
@@ -846,7 +1203,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2F5597"/>
-        <bgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF0563C1"/>
       </patternFill>
     </fill>
     <fill>
@@ -911,7 +1268,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -944,23 +1301,35 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -988,11 +1357,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1020,31 +1389,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1060,7 +1421,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1068,11 +1429,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1084,7 +1445,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1092,7 +1453,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1175,7 +1536,7 @@
       <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0563C1"/>
       <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1394,7 +1755,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:C37"/>
+  <dimension ref="B2:C38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1434,7 +1795,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="5" t="s">
         <v>7</v>
       </c>
@@ -1442,7 +1803,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
         <v>9</v>
       </c>
@@ -1450,7 +1811,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="5" t="s">
         <v>11</v>
       </c>
@@ -1474,19 +1835,19 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="3" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C13" s="6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="B15" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="C15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
@@ -1520,19 +1881,19 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C20" s="6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="6" t="s">
+      <c r="B22" s="3" t="s">
         <v>30</v>
       </c>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="5" t="s">
@@ -1558,7 +1919,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="5" t="s">
         <v>37</v>
       </c>
@@ -1566,19 +1927,19 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="3" t="s">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="4"/>
-    </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="6" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="3" t="s">
         <v>41</v>
       </c>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="5" t="s">
@@ -1596,19 +1957,19 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="3" t="s">
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="4"/>
+      <c r="C32" s="6" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="6" t="s">
+      <c r="B34" s="3" t="s">
         <v>48</v>
       </c>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="5" t="s">
@@ -1626,12 +1987,20 @@
         <v>52</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1646,6 +2015,527 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>171</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I5" r:id="rId1" display="https://www.gpslinkusa.com/"/>
+    <hyperlink ref="I6" r:id="rId2" display="https://ultrongps.com/"/>
+    <hyperlink ref="I7" r:id="rId3" display="https://wolftrakglobal.com/"/>
+    <hyperlink ref="I8" r:id="rId4" display="https://progps.com.do/"/>
+    <hyperlink ref="I9" r:id="rId5" display="https://www.multisolgnp.com/"/>
+    <hyperlink ref="I10" r:id="rId6" display="https://prosecon.tech/es/blog/rastreo-satelital-gps-vehiculos-republica-dominicana"/>
+    <hyperlink ref="I11" r:id="rId7" display="https://gpsgate.com/blog/global-collabs-gpsgate-informac"/>
+    <hyperlink ref="I12" r:id="rId8" display="https://gps.do/inicio/"/>
+    <hyperlink ref="I13" r:id="rId9" display="https://www.geotab.com/es-latam/blog/gestion-de-flotas-caribe/"/>
+    <hyperlink ref="I14" r:id="rId10" display="https://blog.gurtam.com/en/blog/top-20-international-gurtam-partners"/>
+    <hyperlink ref="I15" r:id="rId11" display="https://www.simpliroute.com/es"/>
+    <hyperlink ref="I16" r:id="rId12" display="https://driv.in/"/>
+    <hyperlink ref="I17" r:id="rId13" display="https://www.g2.com/compare/optimoroute-vs-routific"/>
+    <hyperlink ref="I18" r:id="rId14" display="https://motoconchord.org/"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1663,350 +2553,350 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>57</v>
+        <v>174</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>58</v>
+        <v>175</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>59</v>
+        <v>176</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>60</v>
+        <v>177</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>61</v>
+        <v>178</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>62</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="11" t="n">
+      <c r="B5" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>66</v>
+      <c r="E5" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D6" s="11" t="n">
+      <c r="B6" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>69</v>
+      <c r="E6" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" s="11" t="n">
+      <c r="B7" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D7" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>69</v>
+      <c r="E7" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D8" s="11" t="n">
+      <c r="B8" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="D8" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E8" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>69</v>
+      <c r="E8" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="11" t="n">
+      <c r="B9" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>66</v>
+      <c r="E9" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D10" s="11" t="n">
+      <c r="B10" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>79</v>
+      <c r="E10" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="11" t="n">
+      <c r="B11" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D11" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E11" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>66</v>
+      <c r="E11" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="D12" s="11" t="n">
+      <c r="B12" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="D12" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>79</v>
+      <c r="E12" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="11" t="n">
+      <c r="B13" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="D13" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>79</v>
+      <c r="E13" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="D14" s="11" t="n">
+      <c r="B14" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="D14" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E14" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>66</v>
+      <c r="E14" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="D15" s="11" t="n">
+      <c r="B15" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="D15" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E15" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>66</v>
+      <c r="E15" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="n">
+      <c r="A16" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="D16" s="11" t="n">
+      <c r="B16" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="D16" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="E16" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>66</v>
+      <c r="E16" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="n">
+      <c r="A17" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="D17" s="11" t="n">
+      <c r="B17" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D17" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="E17" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>66</v>
+      <c r="E17" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="n">
+      <c r="A18" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="11" t="n">
+      <c r="B18" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="D18" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E18" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>66</v>
+      <c r="E18" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="n">
+      <c r="A19" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="D19" s="11" t="n">
+      <c r="B19" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D19" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E19" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>66</v>
+      <c r="E19" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="C20" s="14" t="str">
+      <c r="B20" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="C20" s="17" t="str">
         <f aca="false">IF(D20=100,"Correcto: suma 100","Revisa: los pesos deben sumar 100")</f>
         <v>Correcto: suma 100</v>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="D20" s="18" t="n">
         <f aca="false">SUM(D5:D19)</f>
         <v>100</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>99</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -2039,7 +2929,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2055,537 +2945,537 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>101</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>58</v>
+        <v>175</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>60</v>
+        <v>177</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>102</v>
+        <v>218</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>108</v>
+        <v>219</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="str">
+      <c r="A5" s="9" t="str">
         <f aca="false">Criterios!B5</f>
         <v>Seguimiento en vivo</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="20" t="n">
         <f aca="false">Criterios!D5</f>
         <v>9</v>
       </c>
-      <c r="C5" s="18" t="str">
+      <c r="C5" s="21" t="str">
         <f aca="false">Criterios!E5</f>
         <v>No</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="str">
+      <c r="A6" s="9" t="str">
         <f aca="false">Criterios!B6</f>
         <v>Geocercas y alertas configurables</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">Criterios!D6</f>
         <v>7</v>
       </c>
-      <c r="C6" s="18" t="str">
+      <c r="C6" s="21" t="str">
         <f aca="false">Criterios!E6</f>
         <v>No</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="str">
+      <c r="A7" s="9" t="str">
         <f aca="false">Criterios!B7</f>
         <v>Historial y reportes</v>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="20" t="n">
         <f aca="false">Criterios!D7</f>
         <v>7</v>
       </c>
-      <c r="C7" s="18" t="str">
+      <c r="C7" s="21" t="str">
         <f aca="false">Criterios!E7</f>
         <v>No</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="str">
+      <c r="A8" s="9" t="str">
         <f aca="false">Criterios!B8</f>
         <v>Cobertura y fiabilidad en nuestras zonas</v>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="20" t="n">
         <f aca="false">Criterios!D8</f>
         <v>7</v>
       </c>
-      <c r="C8" s="18" t="str">
+      <c r="C8" s="21" t="str">
         <f aca="false">Criterios!E8</f>
         <v>Sí</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="str">
+      <c r="A9" s="9" t="str">
         <f aca="false">Criterios!B9</f>
         <v>Funciona con motos</v>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="20" t="n">
         <f aca="false">Criterios!D9</f>
         <v>5</v>
       </c>
-      <c r="C9" s="18" t="str">
+      <c r="C9" s="21" t="str">
         <f aca="false">Criterios!E9</f>
         <v>No</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="str">
+      <c r="A10" s="9" t="str">
         <f aca="false">Criterios!B10</f>
         <v>Planificación de rutas con ventanas de tiempo</v>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="20" t="n">
         <f aca="false">Criterios!D10</f>
         <v>7</v>
       </c>
-      <c r="C10" s="18" t="str">
+      <c r="C10" s="21" t="str">
         <f aca="false">Criterios!E10</f>
         <v>No</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="str">
+      <c r="A11" s="9" t="str">
         <f aca="false">Criterios!B11</f>
         <v>App del conductor en español y simple</v>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="20" t="n">
         <f aca="false">Criterios!D11</f>
         <v>7</v>
       </c>
-      <c r="C11" s="18" t="str">
+      <c r="C11" s="21" t="str">
         <f aca="false">Criterios!E11</f>
         <v>Sí</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="str">
+      <c r="A12" s="9" t="str">
         <f aca="false">Criterios!B12</f>
         <v>Prueba de entrega y estado de paradas</v>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="20" t="n">
         <f aca="false">Criterios!D12</f>
         <v>4</v>
       </c>
-      <c r="C12" s="18" t="str">
+      <c r="C12" s="21" t="str">
         <f aca="false">Criterios!E12</f>
         <v>No</v>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="str">
+      <c r="A13" s="9" t="str">
         <f aca="false">Criterios!B13</f>
         <v>Hora estimada y aviso al cliente</v>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="20" t="n">
         <f aca="false">Criterios!D13</f>
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="str">
+      <c r="C13" s="21" t="str">
         <f aca="false">Criterios!E13</f>
         <v>No</v>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="str">
+      <c r="A14" s="9" t="str">
         <f aca="false">Criterios!B14</f>
         <v>Exportar datos</v>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="20" t="n">
         <f aca="false">Criterios!D14</f>
         <v>7</v>
       </c>
-      <c r="C14" s="18" t="str">
+      <c r="C14" s="21" t="str">
         <f aca="false">Criterios!E14</f>
         <v>Sí</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="str">
+      <c r="A15" s="9" t="str">
         <f aca="false">Criterios!B15</f>
         <v>Facilidad de uso para el supervisor</v>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="20" t="n">
         <f aca="false">Criterios!D15</f>
         <v>7</v>
       </c>
-      <c r="C15" s="18" t="str">
+      <c r="C15" s="21" t="str">
         <f aca="false">Criterios!E15</f>
         <v>No</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="str">
+      <c r="A16" s="9" t="str">
         <f aca="false">Criterios!B16</f>
         <v>Costo total</v>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="20" t="n">
         <f aca="false">Criterios!D16</f>
         <v>12</v>
       </c>
-      <c r="C16" s="18" t="str">
+      <c r="C16" s="21" t="str">
         <f aca="false">Criterios!E16</f>
         <v>No</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="str">
+      <c r="A17" s="9" t="str">
         <f aca="false">Criterios!B17</f>
         <v>Soporte local en español</v>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="20" t="n">
         <f aca="false">Criterios!D17</f>
         <v>8</v>
       </c>
-      <c r="C17" s="18" t="str">
+      <c r="C17" s="21" t="str">
         <f aca="false">Criterios!E17</f>
         <v>Sí</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="str">
+      <c r="A18" s="9" t="str">
         <f aca="false">Criterios!B18</f>
         <v>Contrato y salida</v>
       </c>
-      <c r="B18" s="17" t="n">
+      <c r="B18" s="20" t="n">
         <f aca="false">Criterios!D18</f>
         <v>5</v>
       </c>
-      <c r="C18" s="18" t="str">
+      <c r="C18" s="21" t="str">
         <f aca="false">Criterios!E18</f>
         <v>No</v>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D18" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="str">
+      <c r="A19" s="9" t="str">
         <f aca="false">Criterios!B19</f>
         <v>Privacidad y seguridad de datos</v>
       </c>
-      <c r="B19" s="17" t="n">
+      <c r="B19" s="20" t="n">
         <f aca="false">Criterios!D19</f>
         <v>5</v>
       </c>
-      <c r="C19" s="18" t="str">
+      <c r="C19" s="21" t="str">
         <f aca="false">Criterios!E19</f>
         <v>No</v>
       </c>
-      <c r="D19" s="19" t="n">
+      <c r="D19" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="23" t="n">
+      <c r="A21" s="24" t="s">
+        <v>225</v>
+      </c>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="26" t="n">
         <f aca="false">IF(SUMPRODUCT($B$5:$B$19*(D5:D19&lt;&gt;""))=0,"",SUMPRODUCT($B$5:$B$19*(D5:D19&lt;&gt;"")*D5:D19)/(5*SUMPRODUCT($B$5:$B$19*(D5:D19&lt;&gt;"")))*100)</f>
         <v>74.8</v>
       </c>
-      <c r="E21" s="23" t="str">
+      <c r="E21" s="26" t="str">
         <f aca="false">IF(SUMPRODUCT($B$5:$B$19*(E5:E19&lt;&gt;""))=0,"",SUMPRODUCT($B$5:$B$19*(E5:E19&lt;&gt;"")*E5:E19)/(5*SUMPRODUCT($B$5:$B$19*(E5:E19&lt;&gt;"")))*100)</f>
         <v/>
       </c>
-      <c r="F21" s="23" t="str">
+      <c r="F21" s="26" t="str">
         <f aca="false">IF(SUMPRODUCT($B$5:$B$19*(F5:F19&lt;&gt;""))=0,"",SUMPRODUCT($B$5:$B$19*(F5:F19&lt;&gt;"")*F5:F19)/(5*SUMPRODUCT($B$5:$B$19*(F5:F19&lt;&gt;"")))*100)</f>
         <v/>
       </c>
-      <c r="G21" s="23" t="str">
+      <c r="G21" s="26" t="str">
         <f aca="false">IF(SUMPRODUCT($B$5:$B$19*(G5:G19&lt;&gt;""))=0,"",SUMPRODUCT($B$5:$B$19*(G5:G19&lt;&gt;"")*G5:G19)/(5*SUMPRODUCT($B$5:$B$19*(G5:G19&lt;&gt;"")))*100)</f>
         <v/>
       </c>
-      <c r="H21" s="23" t="str">
+      <c r="H21" s="26" t="str">
         <f aca="false">IF(SUMPRODUCT($B$5:$B$19*(H5:H19&lt;&gt;""))=0,"",SUMPRODUCT($B$5:$B$19*(H5:H19&lt;&gt;"")*H5:H19)/(5*SUMPRODUCT($B$5:$B$19*(H5:H19&lt;&gt;"")))*100)</f>
         <v/>
       </c>
-      <c r="I21" s="23" t="str">
+      <c r="I21" s="26" t="str">
         <f aca="false">IF(SUMPRODUCT($B$5:$B$19*(I5:I19&lt;&gt;""))=0,"",SUMPRODUCT($B$5:$B$19*(I5:I19&lt;&gt;"")*I5:I19)/(5*SUMPRODUCT($B$5:$B$19*(I5:I19&lt;&gt;"")))*100)</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="24" t="s">
-        <v>111</v>
-      </c>
-      <c r="E22" s="25" t="str">
+      <c r="A22" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="27" t="s">
+        <v>227</v>
+      </c>
+      <c r="E22" s="28" t="str">
         <f aca="false">IF(E24="Evaluado",1+COUNTIFS($E$24:$I$24,"Evaluado",$E$21:$I$21,"&gt;"&amp;E21),"-")</f>
         <v>-</v>
       </c>
-      <c r="F22" s="25" t="str">
+      <c r="F22" s="28" t="str">
         <f aca="false">IF(F24="Evaluado",1+COUNTIFS($E$24:$I$24,"Evaluado",$E$21:$I$21,"&gt;"&amp;F21),"-")</f>
         <v>-</v>
       </c>
-      <c r="G22" s="25" t="str">
+      <c r="G22" s="28" t="str">
         <f aca="false">IF(G24="Evaluado",1+COUNTIFS($E$24:$I$24,"Evaluado",$E$21:$I$21,"&gt;"&amp;G21),"-")</f>
         <v>-</v>
       </c>
-      <c r="H22" s="25" t="str">
+      <c r="H22" s="28" t="str">
         <f aca="false">IF(H24="Evaluado",1+COUNTIFS($E$24:$I$24,"Evaluado",$E$21:$I$21,"&gt;"&amp;H21),"-")</f>
         <v>-</v>
       </c>
-      <c r="I22" s="25" t="str">
+      <c r="I22" s="28" t="str">
         <f aca="false">IF(I24="Evaluado",1+COUNTIFS($E$24:$I$24,"Evaluado",$E$21:$I$21,"&gt;"&amp;I21),"-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="18" t="n">
+      <c r="A23" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="21" t="n">
         <f aca="false">COUNTBLANK(D5:D19)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="18" t="n">
+      <c r="E23" s="21" t="n">
         <f aca="false">COUNTBLANK(E5:E19)</f>
         <v>15</v>
       </c>
-      <c r="F23" s="18" t="n">
+      <c r="F23" s="21" t="n">
         <f aca="false">COUNTBLANK(F5:F19)</f>
         <v>15</v>
       </c>
-      <c r="G23" s="18" t="n">
+      <c r="G23" s="21" t="n">
         <f aca="false">COUNTBLANK(G5:G19)</f>
         <v>15</v>
       </c>
-      <c r="H23" s="18" t="n">
+      <c r="H23" s="21" t="n">
         <f aca="false">COUNTBLANK(H5:H19)</f>
         <v>15</v>
       </c>
-      <c r="I23" s="18" t="n">
+      <c r="I23" s="21" t="n">
         <f aca="false">COUNTBLANK(I5:I19)</f>
         <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="25" t="str">
+      <c r="A24" s="24" t="s">
+        <v>229</v>
+      </c>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="28" t="str">
         <f aca="false">IF(D23=15,"Sin datos",IF(SUMPRODUCT(($C$5:$C$19="Sí")*(D5:D19&lt;&gt;"")*(D5:D19&lt;=2))&gt;0,"Descartado",IF(D23&gt;0,"Incompleto","Evaluado")))</f>
         <v>Evaluado</v>
       </c>
-      <c r="E24" s="25" t="str">
+      <c r="E24" s="28" t="str">
         <f aca="false">IF(E23=15,"Sin datos",IF(SUMPRODUCT(($C$5:$C$19="Sí")*(E5:E19&lt;&gt;"")*(E5:E19&lt;=2))&gt;0,"Descartado",IF(E23&gt;0,"Incompleto","Evaluado")))</f>
         <v>Sin datos</v>
       </c>
-      <c r="F24" s="25" t="str">
+      <c r="F24" s="28" t="str">
         <f aca="false">IF(F23=15,"Sin datos",IF(SUMPRODUCT(($C$5:$C$19="Sí")*(F5:F19&lt;&gt;"")*(F5:F19&lt;=2))&gt;0,"Descartado",IF(F23&gt;0,"Incompleto","Evaluado")))</f>
         <v>Sin datos</v>
       </c>
-      <c r="G24" s="25" t="str">
+      <c r="G24" s="28" t="str">
         <f aca="false">IF(G23=15,"Sin datos",IF(SUMPRODUCT(($C$5:$C$19="Sí")*(G5:G19&lt;&gt;"")*(G5:G19&lt;=2))&gt;0,"Descartado",IF(G23&gt;0,"Incompleto","Evaluado")))</f>
         <v>Sin datos</v>
       </c>
-      <c r="H24" s="25" t="str">
+      <c r="H24" s="28" t="str">
         <f aca="false">IF(H23=15,"Sin datos",IF(SUMPRODUCT(($C$5:$C$19="Sí")*(H5:H19&lt;&gt;"")*(H5:H19&lt;=2))&gt;0,"Descartado",IF(H23&gt;0,"Incompleto","Evaluado")))</f>
         <v>Sin datos</v>
       </c>
-      <c r="I24" s="25" t="str">
+      <c r="I24" s="28" t="str">
         <f aca="false">IF(I23=15,"Sin datos",IF(SUMPRODUCT(($C$5:$C$19="Sí")*(I5:I19&lt;&gt;"")*(I5:I19&lt;=2))&gt;0,"Descartado",IF(I23&gt;0,"Incompleto","Evaluado")))</f>
         <v>Sin datos</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B25" s="26" t="n">
+        <v>214</v>
+      </c>
+      <c r="B25" s="29" t="n">
         <f aca="false">SUM(B5:B19)</f>
         <v>100</v>
       </c>
-      <c r="C25" s="27" t="str">
+      <c r="C25" s="30" t="str">
         <f aca="false">IF(B25=100,"","Los pesos no suman 100: corrige en Criterios")</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="28" t="s">
-        <v>114</v>
+      <c r="A27" s="11" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="s">
-        <v>115</v>
+      <c r="A28" s="12" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
-        <v>116</v>
+      <c r="A29" s="12" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="s">
-        <v>117</v>
+      <c r="A30" s="12" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29" t="s">
-        <v>118</v>
+      <c r="A31" s="12" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29" t="s">
-        <v>119</v>
+      <c r="A32" s="12" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -2621,7 +3511,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2635,325 +3525,325 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>121</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="30" t="n">
+      <c r="A4" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="B4" s="31" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>124</v>
+      <c r="A5" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>125</v>
+        <v>241</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="16" t="str">
+        <v>219</v>
+      </c>
+      <c r="C7" s="19" t="str">
         <f aca="false">Evaluación!E4</f>
         <v>Proveedor A</v>
       </c>
-      <c r="D7" s="16" t="str">
+      <c r="D7" s="19" t="str">
         <f aca="false">Evaluación!F4</f>
         <v>Proveedor B</v>
       </c>
-      <c r="E7" s="16" t="str">
+      <c r="E7" s="19" t="str">
         <f aca="false">Evaluación!G4</f>
         <v>Proveedor C</v>
       </c>
-      <c r="F7" s="16" t="str">
+      <c r="F7" s="19" t="str">
         <f aca="false">Evaluación!H4</f>
         <v>Proveedor D</v>
       </c>
-      <c r="G7" s="16" t="str">
+      <c r="G7" s="19" t="str">
         <f aca="false">Evaluación!I4</f>
         <v>Proveedor E</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" s="32" t="n">
+      <c r="A8" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="B8" s="33" t="n">
         <v>3500</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="B9" s="32" t="n">
+      <c r="A9" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="B9" s="33" t="n">
         <v>800</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="B10" s="32" t="n">
+      <c r="A10" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="B10" s="33" t="n">
         <v>650</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="B11" s="32" t="n">
+      <c r="A11" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="B11" s="33" t="n">
         <v>2000</v>
       </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="33"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="B12" s="32" t="n">
+      <c r="A12" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="B12" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="B13" s="34" t="n">
+      <c r="A13" s="24" t="s">
+        <v>247</v>
+      </c>
+      <c r="B13" s="35" t="n">
         <f aca="false">IF(COUNT(B8:B11)&lt;4,"",$B$4*(B8+B9))</f>
         <v>103200</v>
       </c>
-      <c r="C13" s="35" t="str">
+      <c r="C13" s="36" t="str">
         <f aca="false">IF(COUNT(C8:C11)&lt;4,"",$B$4*(C8+C9))</f>
         <v/>
       </c>
-      <c r="D13" s="35" t="str">
+      <c r="D13" s="36" t="str">
         <f aca="false">IF(COUNT(D8:D11)&lt;4,"",$B$4*(D8+D9))</f>
         <v/>
       </c>
-      <c r="E13" s="35" t="str">
+      <c r="E13" s="36" t="str">
         <f aca="false">IF(COUNT(E8:E11)&lt;4,"",$B$4*(E8+E9))</f>
         <v/>
       </c>
-      <c r="F13" s="35" t="str">
+      <c r="F13" s="36" t="str">
         <f aca="false">IF(COUNT(F8:F11)&lt;4,"",$B$4*(F8+F9))</f>
         <v/>
       </c>
-      <c r="G13" s="35" t="str">
+      <c r="G13" s="36" t="str">
         <f aca="false">IF(COUNT(G8:G11)&lt;4,"",$B$4*(G8+G9))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="B14" s="34" t="n">
+      <c r="A14" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="B14" s="35" t="n">
         <f aca="false">IF(COUNT(B8:B11)&lt;4,"",$B$4*B10+B11)</f>
         <v>17600</v>
       </c>
-      <c r="C14" s="35" t="str">
+      <c r="C14" s="36" t="str">
         <f aca="false">IF(COUNT(C8:C11)&lt;4,"",$B$4*C10+C11)</f>
         <v/>
       </c>
-      <c r="D14" s="35" t="str">
+      <c r="D14" s="36" t="str">
         <f aca="false">IF(COUNT(D8:D11)&lt;4,"",$B$4*D10+D11)</f>
         <v/>
       </c>
-      <c r="E14" s="35" t="str">
+      <c r="E14" s="36" t="str">
         <f aca="false">IF(COUNT(E8:E11)&lt;4,"",$B$4*E10+E11)</f>
         <v/>
       </c>
-      <c r="F14" s="35" t="str">
+      <c r="F14" s="36" t="str">
         <f aca="false">IF(COUNT(F8:F11)&lt;4,"",$B$4*F10+F11)</f>
         <v/>
       </c>
-      <c r="G14" s="35" t="str">
+      <c r="G14" s="36" t="str">
         <f aca="false">IF(COUNT(G8:G11)&lt;4,"",$B$4*G10+G11)</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="B15" s="34" t="n">
+      <c r="A15" s="24" t="s">
+        <v>249</v>
+      </c>
+      <c r="B15" s="35" t="n">
         <f aca="false">IF(B13="","",B13+12*B14)</f>
         <v>314400</v>
       </c>
-      <c r="C15" s="35" t="str">
+      <c r="C15" s="36" t="str">
         <f aca="false">IF(C13="","",C13+12*C14)</f>
         <v/>
       </c>
-      <c r="D15" s="35" t="str">
+      <c r="D15" s="36" t="str">
         <f aca="false">IF(D13="","",D13+12*D14)</f>
         <v/>
       </c>
-      <c r="E15" s="35" t="str">
+      <c r="E15" s="36" t="str">
         <f aca="false">IF(E13="","",E13+12*E14)</f>
         <v/>
       </c>
-      <c r="F15" s="35" t="str">
+      <c r="F15" s="36" t="str">
         <f aca="false">IF(F13="","",F13+12*F14)</f>
         <v/>
       </c>
-      <c r="G15" s="35" t="str">
+      <c r="G15" s="36" t="str">
         <f aca="false">IF(G13="","",G13+12*G14)</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="B16" s="34" t="n">
+      <c r="A16" s="24" t="s">
+        <v>250</v>
+      </c>
+      <c r="B16" s="35" t="n">
         <f aca="false">IF(B13="","",B13+24*B14)</f>
         <v>525600</v>
       </c>
-      <c r="C16" s="35" t="str">
+      <c r="C16" s="36" t="str">
         <f aca="false">IF(C13="","",C13+24*C14)</f>
         <v/>
       </c>
-      <c r="D16" s="35" t="str">
+      <c r="D16" s="36" t="str">
         <f aca="false">IF(D13="","",D13+24*D14)</f>
         <v/>
       </c>
-      <c r="E16" s="35" t="str">
+      <c r="E16" s="36" t="str">
         <f aca="false">IF(E13="","",E13+24*E14)</f>
         <v/>
       </c>
-      <c r="F16" s="35" t="str">
+      <c r="F16" s="36" t="str">
         <f aca="false">IF(F13="","",F13+24*F14)</f>
         <v/>
       </c>
-      <c r="G16" s="35" t="str">
+      <c r="G16" s="36" t="str">
         <f aca="false">IF(G13="","",G13+24*G14)</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="B17" s="34" t="n">
+      <c r="A17" s="24" t="s">
+        <v>251</v>
+      </c>
+      <c r="B17" s="35" t="n">
         <f aca="false">IF(B16="","",B16/(24*$B$4))</f>
         <v>912.5</v>
       </c>
-      <c r="C17" s="35" t="str">
+      <c r="C17" s="36" t="str">
         <f aca="false">IF(C16="","",C16/(24*$B$4))</f>
         <v/>
       </c>
-      <c r="D17" s="35" t="str">
+      <c r="D17" s="36" t="str">
         <f aca="false">IF(D16="","",D16/(24*$B$4))</f>
         <v/>
       </c>
-      <c r="E17" s="35" t="str">
+      <c r="E17" s="36" t="str">
         <f aca="false">IF(E16="","",E16/(24*$B$4))</f>
         <v/>
       </c>
-      <c r="F17" s="35" t="str">
+      <c r="F17" s="36" t="str">
         <f aca="false">IF(F16="","",F16/(24*$B$4))</f>
         <v/>
       </c>
-      <c r="G17" s="35" t="str">
+      <c r="G17" s="36" t="str">
         <f aca="false">IF(G16="","",G16/(24*$B$4))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="B18" s="34" t="n">
+      <c r="A18" s="24" t="s">
+        <v>252</v>
+      </c>
+      <c r="B18" s="35" t="n">
         <f aca="false">IF(OR(B12="",B14=""),"",B13+B12*B14)</f>
         <v>314400</v>
       </c>
-      <c r="C18" s="35" t="str">
+      <c r="C18" s="36" t="str">
         <f aca="false">IF(OR(C12="",C14=""),"",C13+C12*C14)</f>
         <v/>
       </c>
-      <c r="D18" s="35" t="str">
+      <c r="D18" s="36" t="str">
         <f aca="false">IF(OR(D12="",D14=""),"",D13+D12*D14)</f>
         <v/>
       </c>
-      <c r="E18" s="35" t="str">
+      <c r="E18" s="36" t="str">
         <f aca="false">IF(OR(E12="",E14=""),"",E13+E12*E14)</f>
         <v/>
       </c>
-      <c r="F18" s="35" t="str">
+      <c r="F18" s="36" t="str">
         <f aca="false">IF(OR(F12="",F14=""),"",F13+F12*F14)</f>
         <v/>
       </c>
-      <c r="G18" s="35" t="str">
+      <c r="G18" s="36" t="str">
         <f aca="false">IF(OR(G12="",G14=""),"",G13+G12*G14)</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
-        <v>137</v>
+      <c r="A20" s="11" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29" t="s">
-        <v>138</v>
+      <c r="A21" s="12" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="s">
-        <v>139</v>
+      <c r="A22" s="12" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29" t="s">
-        <v>140</v>
+      <c r="A23" s="12" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29" t="s">
-        <v>141</v>
+      <c r="A24" s="12" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="s">
-        <v>142</v>
+      <c r="A25" s="12" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -2967,7 +3857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2983,302 +3873,302 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>144</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>145</v>
+        <v>261</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>146</v>
+        <v>262</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="D4" s="16" t="str">
+        <v>263</v>
+      </c>
+      <c r="D4" s="19" t="str">
         <f aca="false">Evaluación!E4</f>
         <v>Proveedor A</v>
       </c>
-      <c r="E4" s="16" t="str">
+      <c r="E4" s="19" t="str">
         <f aca="false">Evaluación!F4</f>
         <v>Proveedor B</v>
       </c>
-      <c r="F4" s="16" t="str">
+      <c r="F4" s="19" t="str">
         <f aca="false">Evaluación!G4</f>
         <v>Proveedor C</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="C5" s="36" t="s">
-        <v>150</v>
-      </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="A5" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="C6" s="36" t="s">
-        <v>152</v>
-      </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
+      <c r="A6" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="C6" s="37" t="s">
+        <v>268</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="C7" s="36" t="s">
-        <v>154</v>
-      </c>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
+      <c r="A7" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>270</v>
+      </c>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="C8" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
+      <c r="A8" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="C8" s="37" t="s">
+        <v>272</v>
+      </c>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
+      <c r="A9" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="C9" s="37" t="s">
+        <v>275</v>
+      </c>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>161</v>
-      </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
+      <c r="A10" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="C10" s="37" t="s">
+        <v>277</v>
+      </c>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="C11" s="36" t="s">
-        <v>163</v>
-      </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
+      <c r="A11" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>279</v>
+      </c>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="C12" s="36" t="s">
-        <v>165</v>
-      </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
+      <c r="A12" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="C12" s="37" t="s">
+        <v>281</v>
+      </c>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>167</v>
-      </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
+      <c r="A13" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>283</v>
+      </c>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="C14" s="36" t="s">
-        <v>170</v>
-      </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="A14" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>286</v>
+      </c>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="C15" s="36" t="s">
-        <v>172</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
+      <c r="A15" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="C15" s="37" t="s">
+        <v>288</v>
+      </c>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="C16" s="36" t="s">
-        <v>175</v>
-      </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
+      <c r="A16" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="C16" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="C17" s="36" t="s">
-        <v>177</v>
-      </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
+      <c r="A17" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="C17" s="37" t="s">
+        <v>293</v>
+      </c>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="C18" s="36" t="s">
-        <v>179</v>
-      </c>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
+      <c r="A18" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="C18" s="37" t="s">
+        <v>295</v>
+      </c>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="C19" s="36" t="s">
-        <v>182</v>
-      </c>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
+      <c r="A19" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>298</v>
+      </c>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="C20" s="36" t="s">
-        <v>184</v>
-      </c>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
+      <c r="A20" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="C20" s="37" t="s">
+        <v>300</v>
+      </c>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="C21" s="36" t="s">
-        <v>186</v>
-      </c>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
+      <c r="A21" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="C22" s="36" t="s">
-        <v>188</v>
-      </c>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
+      <c r="A22" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>304</v>
+      </c>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="C23" s="36" t="s">
-        <v>191</v>
-      </c>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="A23" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3291,7 +4181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3309,325 +4199,325 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B4" s="31"/>
+      <c r="A4" s="16" t="s">
+        <v>310</v>
+      </c>
+      <c r="B4" s="32"/>
       <c r="C4" s="2" t="s">
-        <v>195</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="B5" s="31"/>
+      <c r="A5" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="B5" s="32"/>
       <c r="C5" s="2" t="s">
-        <v>197</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="B6" s="37"/>
+      <c r="A6" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="B6" s="38"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="B7" s="37"/>
+      <c r="A7" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="B8" s="31"/>
+      <c r="A8" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="B8" s="32"/>
       <c r="C8" s="2" t="s">
-        <v>201</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>202</v>
+        <v>318</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>203</v>
+        <v>319</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>204</v>
+        <v>320</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>205</v>
+        <v>321</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>206</v>
+        <v>322</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>207</v>
+        <v>323</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>208</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
-        <v>209</v>
-      </c>
-      <c r="B11" s="39" t="s">
-        <v>210</v>
-      </c>
-      <c r="C11" s="40" t="n">
+      <c r="A11" s="39" t="s">
+        <v>325</v>
+      </c>
+      <c r="B11" s="40" t="s">
+        <v>326</v>
+      </c>
+      <c r="C11" s="41" t="n">
         <v>40</v>
       </c>
-      <c r="D11" s="40" t="n">
+      <c r="D11" s="41" t="n">
         <v>22</v>
       </c>
-      <c r="E11" s="41" t="n">
+      <c r="E11" s="42" t="n">
         <f aca="false">IF(OR(C11="",D11="",C11=0),"",(D11-C11)/C11)</f>
         <v>-0.45</v>
       </c>
-      <c r="F11" s="42" t="str">
+      <c r="F11" s="43" t="str">
         <f aca="false">IF(OR(C11="",D11=""),"",IF(D11=C11,"Igual",IF(OR(AND(B11="Baja",D11&lt;C11),AND(B11="Sube",D11&gt;C11)),"Mejoró","Empeoró")))</f>
         <v>Mejoró</v>
       </c>
-      <c r="G11" s="36" t="s">
-        <v>211</v>
+      <c r="G11" s="37" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="41" t="str">
+      <c r="A12" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="42" t="str">
         <f aca="false">IF(OR(C12="",D12="",C12=0),"",(D12-C12)/C12)</f>
         <v/>
       </c>
-      <c r="F12" s="42" t="str">
+      <c r="F12" s="43" t="str">
         <f aca="false">IF(OR(C12="",D12=""),"",IF(D12=C12,"Igual",IF(OR(AND(B12="Baja",D12&lt;C12),AND(B12="Sube",D12&gt;C12)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G12" s="36" t="s">
-        <v>213</v>
+      <c r="G12" s="37" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="41" t="str">
+      <c r="A13" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="42" t="str">
         <f aca="false">IF(OR(C13="",D13="",C13=0),"",(D13-C13)/C13)</f>
         <v/>
       </c>
-      <c r="F13" s="42" t="str">
+      <c r="F13" s="43" t="str">
         <f aca="false">IF(OR(C13="",D13=""),"",IF(D13=C13,"Igual",IF(OR(AND(B13="Baja",D13&lt;C13),AND(B13="Sube",D13&gt;C13)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G13" s="36" t="s">
-        <v>215</v>
+      <c r="G13" s="37" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="41" t="str">
+      <c r="A14" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="42" t="str">
         <f aca="false">IF(OR(C14="",D14="",C14=0),"",(D14-C14)/C14)</f>
         <v/>
       </c>
-      <c r="F14" s="42" t="str">
+      <c r="F14" s="43" t="str">
         <f aca="false">IF(OR(C14="",D14=""),"",IF(D14=C14,"Igual",IF(OR(AND(B14="Baja",D14&lt;C14),AND(B14="Sube",D14&gt;C14)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G14" s="36" t="s">
-        <v>217</v>
+      <c r="G14" s="37" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="41" t="str">
+      <c r="A15" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="42" t="str">
         <f aca="false">IF(OR(C15="",D15="",C15=0),"",(D15-C15)/C15)</f>
         <v/>
       </c>
-      <c r="F15" s="42" t="str">
+      <c r="F15" s="43" t="str">
         <f aca="false">IF(OR(C15="",D15=""),"",IF(D15=C15,"Igual",IF(OR(AND(B15="Baja",D15&lt;C15),AND(B15="Sube",D15&gt;C15)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G15" s="36" t="s">
-        <v>219</v>
+      <c r="G15" s="37" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="C16" s="43"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="41" t="str">
+      <c r="A16" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="42" t="str">
         <f aca="false">IF(OR(C16="",D16="",C16=0),"",(D16-C16)/C16)</f>
         <v/>
       </c>
-      <c r="F16" s="42" t="str">
+      <c r="F16" s="43" t="str">
         <f aca="false">IF(OR(C16="",D16=""),"",IF(D16=C16,"Igual",IF(OR(AND(B16="Baja",D16&lt;C16),AND(B16="Sube",D16&gt;C16)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G16" s="36" t="s">
-        <v>221</v>
+      <c r="G16" s="37" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="41" t="str">
+      <c r="A17" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="42" t="str">
         <f aca="false">IF(OR(C17="",D17="",C17=0),"",(D17-C17)/C17)</f>
         <v/>
       </c>
-      <c r="F17" s="42" t="str">
+      <c r="F17" s="43" t="str">
         <f aca="false">IF(OR(C17="",D17=""),"",IF(D17=C17,"Igual",IF(OR(AND(B17="Baja",D17&lt;C17),AND(B17="Sube",D17&gt;C17)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G17" s="36" t="s">
-        <v>223</v>
+      <c r="G17" s="37" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="41" t="str">
+      <c r="A18" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="42" t="str">
         <f aca="false">IF(OR(C18="",D18="",C18=0),"",(D18-C18)/C18)</f>
         <v/>
       </c>
-      <c r="F18" s="42" t="str">
+      <c r="F18" s="43" t="str">
         <f aca="false">IF(OR(C18="",D18=""),"",IF(D18=C18,"Igual",IF(OR(AND(B18="Baja",D18&lt;C18),AND(B18="Sube",D18&gt;C18)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G18" s="36" t="s">
-        <v>225</v>
+      <c r="G18" s="37" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="41" t="str">
+      <c r="A19" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="42" t="str">
         <f aca="false">IF(OR(C19="",D19="",C19=0),"",(D19-C19)/C19)</f>
         <v/>
       </c>
-      <c r="F19" s="42" t="str">
+      <c r="F19" s="43" t="str">
         <f aca="false">IF(OR(C19="",D19=""),"",IF(D19=C19,"Igual",IF(OR(AND(B19="Baja",D19&lt;C19),AND(B19="Sube",D19&gt;C19)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G19" s="36" t="s">
-        <v>228</v>
+      <c r="G19" s="37" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="41" t="str">
+      <c r="A20" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="42" t="str">
         <f aca="false">IF(OR(C20="",D20="",C20=0),"",(D20-C20)/C20)</f>
         <v/>
       </c>
-      <c r="F20" s="42" t="str">
+      <c r="F20" s="43" t="str">
         <f aca="false">IF(OR(C20="",D20=""),"",IF(D20=C20,"Igual",IF(OR(AND(B20="Baja",D20&lt;C20),AND(B20="Sube",D20&gt;C20)),"Mejoró","Empeoró")))</f>
         <v/>
       </c>
-      <c r="G20" s="36" t="s">
-        <v>230</v>
+      <c r="G20" s="37" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="B22" s="44" t="n">
+      <c r="A22" s="16" t="s">
+        <v>347</v>
+      </c>
+      <c r="B22" s="45" t="n">
         <f aca="false">COUNTIF(F12:F20,"Mejoró")</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="B23" s="44" t="n">
+      <c r="A23" s="16" t="s">
+        <v>348</v>
+      </c>
+      <c r="B23" s="45" t="n">
         <f aca="false">COUNTIF(F12:F20,"Empeoró")</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="B25" s="31"/>
+      <c r="A25" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="B25" s="32"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>234</v>
-      </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
+      <c r="A26" s="16" t="s">
+        <v>350</v>
+      </c>
+      <c r="B26" s="46"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>235</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>